<commit_message>
Spell out every identifier
ACC-1001 is now ACCOUNT-1001, TCK-004417 is TICKET-004417, PRP-000301 is
PROPOSAL-000301, KB-0117 is ARTICLE-0117, and the same for POLICY, INCIDENT,
ESCALATION, REQUEST, ISSUE, OPPORTUNITY, DECISION, EXPERIMENT and BLOCKER.

Person codes are gone entirely. P-LUC is Lucia Ferreira. A name reads better
than a code that has to be looked up, and the code bought nothing.

Word documents and spreadsheets were rewritten at the zip level rather than
through openpyxl or python-docx, so the reporting pack's stale cached value
survived. It was the point of that fixture and a library round-trip would have
destroyed it.

Two things the bulk rename missed and the tests caught: the OpenAPI contract's
regex patterns, where the prefix is followed by a character class rather than a
digit, and two f-strings that generate proposal identifiers at runtime.
</commit_message>
<xml_diff>
--- a/data/packs/pack-template.xlsx
+++ b/data/packs/pack-template.xlsx
@@ -427,14 +427,14 @@
     <row r="3" ht="15" customHeight="1" s="7">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Account: &lt;ACC-NNNN&gt;</t>
+          <t>Account: &lt;ACCOUNT-NNNN&gt;</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="7">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Prepared by: P-LUC</t>
+          <t>Prepared by: Lucia Ferreira</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
     <row r="4" ht="15" customHeight="1" s="7">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>ESC-0409</t>
+          <t>ESCALATION-0409</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">

</xml_diff>